<commit_message>
Implementation of R_SWITCH, the Daq Task has changed the name to R_SWITCH. Bug fix, now the resistance names are forced to be str before being loaded into the Parameter Tree.
New: Two scripts to compare signals.
</commit_message>
<xml_diff>
--- a/ParameterFormat.xlsx
+++ b/ParameterFormat.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmartic\PycharmProjects\pyTENG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9417D87-DCE3-4912-A7BF-86BF276A6C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08CC6811-C48D-47FE-ABC9-85CA26F145BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>NAME</t>
   </si>
@@ -36,12 +36,6 @@
     <t>ATENUATION</t>
   </si>
   <si>
-    <t>Resistance 1</t>
-  </si>
-  <si>
-    <t>Resistance 2</t>
-  </si>
-  <si>
     <t>Resistance 3</t>
   </si>
   <si>
@@ -79,9 +73,6 @@
   </si>
   <si>
     <t>Resistance 15</t>
-  </si>
-  <si>
-    <t>Resistance 0</t>
   </si>
   <si>
     <t>DAQ_CODE</t>
@@ -537,57 +528,57 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>18</v>
+      <c r="A2" s="3">
+        <v>10</v>
       </c>
       <c r="B2" s="3">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C2" s="5">
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F2" s="4"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>3</v>
+      <c r="A3" s="3">
+        <v>50</v>
       </c>
       <c r="B3" s="3">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C3" s="5">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>4</v>
+      <c r="A4" s="3">
+        <v>100</v>
       </c>
       <c r="B4" s="3">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="C4" s="5">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B5" s="3">
         <v>20</v>
@@ -596,13 +587,13 @@
         <v>1.6</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6" s="3">
         <v>25</v>
@@ -611,13 +602,13 @@
         <v>1.8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B7" s="3">
         <v>30</v>
@@ -626,13 +617,13 @@
         <v>2</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B8" s="3">
         <v>35</v>
@@ -641,13 +632,13 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B9" s="3">
         <v>40</v>
@@ -656,13 +647,13 @@
         <v>2.4</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B10" s="3">
         <v>45</v>
@@ -671,13 +662,13 @@
         <v>2.6</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B11" s="3">
         <v>50</v>
@@ -686,13 +677,13 @@
         <v>2.8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B12" s="3">
         <v>55</v>
@@ -701,13 +692,13 @@
         <v>3</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F12" s="4"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B13" s="3">
         <v>60</v>
@@ -716,13 +707,13 @@
         <v>3.2</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B14" s="3">
         <v>65</v>
@@ -731,13 +722,13 @@
         <v>3.4</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B15" s="3">
         <v>70</v>
@@ -746,13 +737,13 @@
         <v>3.6</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F15" s="4"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B16" s="3">
         <v>75</v>
@@ -761,13 +752,13 @@
         <v>3.8</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F16" s="4"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B17" s="3">
         <v>80</v>
@@ -776,13 +767,13 @@
         <v>4</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F17" s="4"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B18" s="3">
         <v>85</v>
@@ -791,13 +782,13 @@
         <v>4.2</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F18" s="4"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B19" s="3">
         <v>90</v>
@@ -806,13 +797,13 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F19" s="4"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B20" s="3">
         <v>95</v>
@@ -821,13 +812,13 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F20" s="4"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B21" s="3">
         <v>100</v>
@@ -836,13 +827,13 @@
         <v>4.8</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F21" s="4"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B22" s="3">
         <v>105</v>
@@ -851,13 +842,13 @@
         <v>5</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F22" s="4"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B23" s="3">
         <v>110</v>
@@ -866,13 +857,13 @@
         <v>5.2</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F23" s="4"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B24" s="3">
         <v>115</v>
@@ -881,13 +872,13 @@
         <v>5.4</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F24" s="4"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B25" s="3">
         <v>120</v>
@@ -896,7 +887,7 @@
         <v>5.6</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F25" s="4"/>
     </row>

</xml_diff>